<commit_message>
fixed last diagramm svg errors
</commit_message>
<xml_diff>
--- a/B.Sc. LRT/Strömungslehre 2/images/SL2-Diagrams.xlsx
+++ b/B.Sc. LRT/Strömungslehre 2/images/SL2-Diagrams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Phillip\Documents\Git\Project-FoSa\B.Sc. LRT\Strömungslehre 2\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D246A5B-C7CC-4EAF-9A6A-5A245F7B72B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E139171B-6CD0-46D3-AD5A-DDE983213783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="18696" activeTab="5" xr2:uid="{FA5394E7-ED4E-4AC0-A8BA-0A137B0856E0}"/>
   </bookViews>
@@ -482,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -558,6 +558,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -585,12 +612,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -599,6 +620,12 @@
     </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -616,36 +643,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -29633,19 +29630,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.4">
-      <c r="B3" s="31"/>
+      <c r="B3" s="42"/>
       <c r="C3" s="6" t="s">
         <v>6</v>
       </c>
@@ -30455,130 +30452,130 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:41" ht="15.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="33" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
-      <c r="T2" s="34"/>
-      <c r="U2" s="34"/>
-      <c r="V2" s="34"/>
-      <c r="W2" s="34"/>
-      <c r="X2" s="34"/>
-      <c r="Y2" s="34"/>
-      <c r="Z2" s="34"/>
-      <c r="AA2" s="34"/>
-      <c r="AB2" s="34"/>
-      <c r="AC2" s="34"/>
-      <c r="AD2" s="34"/>
-      <c r="AE2" s="34"/>
-      <c r="AF2" s="34"/>
-      <c r="AG2" s="34"/>
-      <c r="AH2" s="34"/>
-      <c r="AI2" s="34"/>
-      <c r="AJ2" s="34"/>
-      <c r="AK2" s="34"/>
-      <c r="AL2" s="34"/>
-      <c r="AM2" s="34"/>
-      <c r="AN2" s="34"/>
-      <c r="AO2" s="35"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
+      <c r="AB2" s="45"/>
+      <c r="AC2" s="45"/>
+      <c r="AD2" s="45"/>
+      <c r="AE2" s="45"/>
+      <c r="AF2" s="45"/>
+      <c r="AG2" s="45"/>
+      <c r="AH2" s="45"/>
+      <c r="AI2" s="45"/>
+      <c r="AJ2" s="45"/>
+      <c r="AK2" s="45"/>
+      <c r="AL2" s="45"/>
+      <c r="AM2" s="45"/>
+      <c r="AN2" s="45"/>
+      <c r="AO2" s="46"/>
     </row>
     <row r="3" spans="2:41" ht="15.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="32">
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="43">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32">
+      <c r="E3" s="43"/>
+      <c r="F3" s="43">
         <v>1.2</v>
       </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32">
+      <c r="G3" s="43"/>
+      <c r="H3" s="43">
         <v>1.3</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32">
+      <c r="I3" s="43"/>
+      <c r="J3" s="43">
         <v>1.4</v>
       </c>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32">
+      <c r="K3" s="43"/>
+      <c r="L3" s="43">
         <v>1.5</v>
       </c>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32">
+      <c r="M3" s="43"/>
+      <c r="N3" s="43">
         <v>1.6</v>
       </c>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32">
+      <c r="O3" s="43"/>
+      <c r="P3" s="43">
         <v>1.7</v>
       </c>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32">
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43">
         <v>1.8</v>
       </c>
-      <c r="S3" s="32"/>
-      <c r="T3" s="32">
+      <c r="S3" s="43"/>
+      <c r="T3" s="43">
         <v>1.9</v>
       </c>
-      <c r="U3" s="32"/>
-      <c r="V3" s="32">
+      <c r="U3" s="43"/>
+      <c r="V3" s="43">
         <v>2</v>
       </c>
-      <c r="W3" s="32"/>
-      <c r="X3" s="32">
+      <c r="W3" s="43"/>
+      <c r="X3" s="43">
         <v>2.1</v>
       </c>
-      <c r="Y3" s="32"/>
-      <c r="Z3" s="32">
+      <c r="Y3" s="43"/>
+      <c r="Z3" s="43">
         <v>2.2000000000000002</v>
       </c>
-      <c r="AA3" s="32"/>
-      <c r="AB3" s="32">
+      <c r="AA3" s="43"/>
+      <c r="AB3" s="43">
         <v>2.2999999999999998</v>
       </c>
-      <c r="AC3" s="32"/>
-      <c r="AD3" s="32">
+      <c r="AC3" s="43"/>
+      <c r="AD3" s="43">
         <v>2.4</v>
       </c>
-      <c r="AE3" s="32"/>
-      <c r="AF3" s="32">
+      <c r="AE3" s="43"/>
+      <c r="AF3" s="43">
         <v>3</v>
       </c>
-      <c r="AG3" s="32"/>
-      <c r="AH3" s="32">
+      <c r="AG3" s="43"/>
+      <c r="AH3" s="43">
         <v>4</v>
       </c>
-      <c r="AI3" s="32"/>
-      <c r="AJ3" s="32">
+      <c r="AI3" s="43"/>
+      <c r="AJ3" s="43">
         <v>5</v>
       </c>
-      <c r="AK3" s="32"/>
-      <c r="AL3" s="32">
+      <c r="AK3" s="43"/>
+      <c r="AL3" s="43">
         <v>10</v>
       </c>
-      <c r="AM3" s="32"/>
-      <c r="AN3" s="32">
+      <c r="AM3" s="43"/>
+      <c r="AN3" s="43">
         <v>100000</v>
       </c>
-      <c r="AO3" s="32"/>
+      <c r="AO3" s="43"/>
     </row>
     <row r="4" spans="2:41" ht="15.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="11" t="s">
@@ -31291,7 +31288,7 @@
         <v>-3.9524844257189821E-2</v>
       </c>
       <c r="AG14" s="3">
-        <f t="shared" ref="AE14:AG14" si="22">AF14*180/PI()</f>
+        <f t="shared" ref="AG14" si="22">AF14*180/PI()</f>
         <v>-2.2646067618488663</v>
       </c>
       <c r="AH14" s="3">
@@ -31368,7 +31365,7 @@
         <v>1.3497284394437131E-2</v>
       </c>
       <c r="AG15" s="3">
-        <f t="shared" ref="AE15:AG15" si="27">AF15*180/PI()</f>
+        <f t="shared" ref="AG15" si="27">AF15*180/PI()</f>
         <v>0.7733374306890366</v>
       </c>
       <c r="AH15" s="3">
@@ -31445,7 +31442,7 @@
         <v>6.1691950904027966E-2</v>
       </c>
       <c r="AG16" s="3">
-        <f t="shared" ref="AE16:AG16" si="32">AF16*180/PI()</f>
+        <f t="shared" ref="AG16" si="32">AF16*180/PI()</f>
         <v>3.534688416729086</v>
       </c>
       <c r="AH16" s="3">
@@ -31514,7 +31511,7 @@
       <c r="Z17" s="3"/>
       <c r="AA17" s="3"/>
       <c r="AB17" s="3">
-        <f t="shared" ref="AB9:AB29" si="37">ATAN(_xlfn.COT($C17)*((AB$3^2*(SIN($C17))^2-1)/(1+(((1.4+1)/(2))-(SIN($C17))^2)*AB$3^2)))</f>
+        <f t="shared" ref="AB17:AB29" si="37">ATAN(_xlfn.COT($C17)*((AB$3^2*(SIN($C17))^2-1)/(1+(((1.4+1)/(2))-(SIN($C17))^2)*AB$3^2)))</f>
         <v>-4.3295218683936113E-2</v>
       </c>
       <c r="AC17" s="3">
@@ -31601,7 +31598,7 @@
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3">
-        <f t="shared" ref="F7:AB29" si="44">ATAN(_xlfn.COT($C18)*((Z$3^2*(SIN($C18))^2-1)/(1+(((1.4+1)/(2))-(SIN($C18))^2)*Z$3^2)))</f>
+        <f t="shared" ref="J18:Z29" si="44">ATAN(_xlfn.COT($C18)*((Z$3^2*(SIN($C18))^2-1)/(1+(((1.4+1)/(2))-(SIN($C18))^2)*Z$3^2)))</f>
         <v>-2.4377653264411013E-2</v>
       </c>
       <c r="AA18" s="3">
@@ -32148,7 +32145,7 @@
         <v>-6.0678375318399267E-4</v>
       </c>
       <c r="Q23" s="3">
-        <f t="shared" ref="O23:Q23" si="93">P23*180/PI()</f>
+        <f t="shared" ref="Q23" si="93">P23*180/PI()</f>
         <v>-3.476614813455061E-2</v>
       </c>
       <c r="R23" s="3">
@@ -33540,7 +33537,7 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3">
-        <f t="shared" ref="F31:F50" si="227">ATAN(_xlfn.COT($C33)*((F$3^2*(SIN($C33))^2-1)/(1+(((1.4+1)/(2))-(SIN($C33))^2)*F$3^2)))</f>
+        <f t="shared" ref="F33:F50" si="227">ATAN(_xlfn.COT($C33)*((F$3^2*(SIN($C33))^2-1)/(1+(((1.4+1)/(2))-(SIN($C33))^2)*F$3^2)))</f>
         <v>-3.9902039737076591E-3</v>
       </c>
       <c r="G33" s="3">
@@ -34158,7 +34155,7 @@
         <v>1.1170107212763709</v>
       </c>
       <c r="D37" s="3">
-        <f t="shared" ref="D7:D50" si="276">ATAN(_xlfn.COT($C37)*((D$3^2*(SIN($C37))^2-1)/(1+(((1.4+1)/(2))-(SIN($C37))^2)*D$3^2)))</f>
+        <f t="shared" ref="D37:D50" si="276">ATAN(_xlfn.COT($C37)*((D$3^2*(SIN($C37))^2-1)/(1+(((1.4+1)/(2))-(SIN($C37))^2)*D$3^2)))</f>
         <v>-7.4504540725525929E-3</v>
       </c>
       <c r="E37" s="3">
@@ -36405,6 +36402,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B2:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="AJ3:AK3"/>
     <mergeCell ref="AL3:AM3"/>
     <mergeCell ref="AN3:AO3"/>
@@ -36421,11 +36423,6 @@
     <mergeCell ref="V3:W3"/>
     <mergeCell ref="X3:Y3"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B2:C3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -36448,24 +36445,24 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="31" t="s">
+      <c r="C2" s="48"/>
+      <c r="D2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B3" s="38"/>
-      <c r="C3" s="39"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="50"/>
       <c r="D3" s="7">
         <v>0</v>
       </c>
@@ -36744,7 +36741,7 @@
         <v>0.27925268031909273</v>
       </c>
       <c r="D17" s="5">
-        <f t="shared" ref="D6:D17" si="8">1/SIN($C17)</f>
+        <f t="shared" ref="D17" si="8">1/SIN($C17)</f>
         <v>3.6279552785433005</v>
       </c>
       <c r="E17" s="5"/>
@@ -36808,7 +36805,7 @@
         <v>2.9238044001630876</v>
       </c>
       <c r="E20" s="5">
-        <f t="shared" ref="E18:E58" si="11">0.295785*SQRT((11.4301*COS($C20)+SIN($C20))/(SIN($C20)*(-0.087489*(COS($C20))^2+SIN($C20)*COS($C20)-0.017498)))</f>
+        <f t="shared" ref="E20:E58" si="11">0.295785*SQRT((11.4301*COS($C20)+SIN($C20))/(SIN($C20)*(-0.087489*(COS($C20))^2+SIN($C20)*COS($C20)-0.017498)))</f>
         <v>3.5367613613854618</v>
       </c>
       <c r="F20" s="5"/>
@@ -36858,7 +36855,7 @@
         <v>2.8814331535021172</v>
       </c>
       <c r="F22" s="5">
-        <f t="shared" ref="F18:F56" si="12">0.419913*SQRT((5.67128*COS($C22)+SIN($C22))/(SIN($C22)*(-0.176327*(COS($C22))^2+SIN($C22)*COS($C22)-0.035265)))</f>
+        <f t="shared" ref="F22:F55" si="12">0.419913*SQRT((5.67128*COS($C22)+SIN($C22))/(SIN($C22)*(-0.176327*(COS($C22))^2+SIN($C22)*COS($C22)-0.035265)))</f>
         <v>3.5786169115837394</v>
       </c>
       <c r="G22" s="5"/>
@@ -36914,7 +36911,7 @@
         <v>2.916779482436954</v>
       </c>
       <c r="G24" s="5">
-        <f t="shared" ref="G20:G54" si="13">0.517638*SQRT((3.73205*COS($C24)+SIN($C24))/(SIN($C24)*(-0.267949*(COS($C24))^2+SIN($C24)*COS($C24)-0.05359)))</f>
+        <f t="shared" ref="G24:G53" si="13">0.517638*SQRT((3.73205*COS($C24)+SIN($C24))/(SIN($C24)*(-0.267949*(COS($C24))^2+SIN($C24)*COS($C24)-0.05359)))</f>
         <v>3.7593356451891826</v>
       </c>
       <c r="H24" s="5"/>
@@ -37005,7 +37002,7 @@
         <v>2.7840822535821181</v>
       </c>
       <c r="H27" s="5">
-        <f t="shared" ref="H23:H52" si="14">0.603299*SQRT((2.74748*COS($C27)+SIN($C27))/(SIN($C27)*(-0.36397*(COS($C27))^2+SIN($C27)*COS($C27)-0.072794)))</f>
+        <f t="shared" ref="H27:H52" si="14">0.603299*SQRT((2.74748*COS($C27)+SIN($C27))/(SIN($C27)*(-0.36397*(COS($C27))^2+SIN($C27)*COS($C27)-0.072794)))</f>
         <v>3.623460285234803</v>
       </c>
       <c r="I27" s="5"/>
@@ -37105,7 +37102,7 @@
         <v>2.7479427797822678</v>
       </c>
       <c r="I30" s="5">
-        <f t="shared" ref="I26:I52" si="15">0.682867*SQRT((2.14451*COS($C30)+SIN($C30))/(SIN($C30)*(-0.466308*(COS($C30))^2+SIN($C30)*COS($C30)-0.093262)))</f>
+        <f t="shared" ref="I30:I51" si="15">0.682867*SQRT((2.14451*COS($C30)+SIN($C30))/(SIN($C30)*(-0.466308*(COS($C30))^2+SIN($C30)*COS($C30)-0.093262)))</f>
         <v>3.6347670171920008</v>
       </c>
       <c r="J30" s="5"/>
@@ -37214,7 +37211,7 @@
         <v>2.8095243001456307</v>
       </c>
       <c r="J33" s="5">
-        <f t="shared" ref="J29:J51" si="16">0.759836*SQRT((1.73205*COS($C33)+SIN($C33))/(SIN($C33)*(-0.57735*(COS($C33))^2+SIN($C33)*COS($C33)-0.11547)))</f>
+        <f t="shared" ref="J33:J49" si="16">0.759836*SQRT((1.73205*COS($C33)+SIN($C33))/(SIN($C33)*(-0.57735*(COS($C33))^2+SIN($C33)*COS($C33)-0.11547)))</f>
         <v>3.8221274100068467</v>
       </c>
       <c r="K33" s="5"/>
@@ -37408,7 +37405,7 @@
         <v>2.7331174760389811</v>
       </c>
       <c r="K38" s="5">
-        <f t="shared" ref="K33:K50" si="17">0.836784*SQRT((1.42815*COS($C38)+SIN($C38))/(SIN($C38)*(-0.700208*(COS($C38))^2+SIN($C38)*COS($C38)-0.140042)))</f>
+        <f t="shared" ref="K38:K47" si="17">0.836784*SQRT((1.42815*COS($C38)+SIN($C38))/(SIN($C38)*(-0.700208*(COS($C38))^2+SIN($C38)*COS($C38)-0.140042)))</f>
         <v>3.6253222002571763</v>
       </c>
     </row>
@@ -38207,49 +38204,49 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:29" ht="15.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="56" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="42" t="s">
+      <c r="F2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="42" t="s">
+      <c r="J2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="42" t="s">
+      <c r="L2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="M2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="42" t="s">
+      <c r="N2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="42" t="s">
+      <c r="P2" s="51" t="s">
         <v>2</v>
       </c>
       <c r="Q2" s="6" t="s">
@@ -38257,92 +38254,92 @@
       </c>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.4">
-      <c r="B3" s="46"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="7">
         <v>0</v>
       </c>
-      <c r="D3" s="43"/>
-      <c r="E3" s="40">
+      <c r="D3" s="52"/>
+      <c r="E3" s="54">
         <v>5</v>
       </c>
-      <c r="F3" s="43"/>
-      <c r="G3" s="40">
+      <c r="F3" s="52"/>
+      <c r="G3" s="54">
         <v>10</v>
       </c>
-      <c r="H3" s="43"/>
-      <c r="I3" s="40">
+      <c r="H3" s="52"/>
+      <c r="I3" s="54">
         <v>15</v>
       </c>
-      <c r="J3" s="43"/>
-      <c r="K3" s="40">
+      <c r="J3" s="52"/>
+      <c r="K3" s="54">
         <v>20</v>
       </c>
-      <c r="L3" s="43"/>
-      <c r="M3" s="40">
+      <c r="L3" s="52"/>
+      <c r="M3" s="54">
         <v>25</v>
       </c>
-      <c r="N3" s="43"/>
-      <c r="O3" s="40">
+      <c r="N3" s="52"/>
+      <c r="O3" s="54">
         <v>30</v>
       </c>
-      <c r="P3" s="43"/>
-      <c r="Q3" s="40">
+      <c r="P3" s="52"/>
+      <c r="Q3" s="54">
         <v>35</v>
       </c>
       <c r="AC3"/>
     </row>
     <row r="4" spans="2:29" x14ac:dyDescent="0.4">
-      <c r="B4" s="46"/>
+      <c r="B4" s="57"/>
       <c r="C4" s="8">
         <f>C3*PI()/180</f>
         <v>0</v>
       </c>
-      <c r="D4" s="43"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="43"/>
-      <c r="K4" s="41"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="43"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="43"/>
-      <c r="Q4" s="41"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="52"/>
+      <c r="M4" s="55"/>
+      <c r="N4" s="52"/>
+      <c r="O4" s="55"/>
+      <c r="P4" s="52"/>
+      <c r="Q4" s="55"/>
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.4">
-      <c r="B5" s="47"/>
+      <c r="B5" s="58"/>
       <c r="C5" s="14">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
-      <c r="D5" s="44"/>
+      <c r="D5" s="53"/>
       <c r="E5" s="15">
         <v>1.5</v>
       </c>
-      <c r="F5" s="44"/>
+      <c r="F5" s="53"/>
       <c r="G5" s="15">
         <v>1.46</v>
       </c>
-      <c r="H5" s="44"/>
+      <c r="H5" s="53"/>
       <c r="I5" s="15">
         <v>1.42</v>
       </c>
-      <c r="J5" s="44"/>
+      <c r="J5" s="53"/>
       <c r="K5" s="23">
         <v>1.39</v>
       </c>
-      <c r="L5" s="44"/>
+      <c r="L5" s="53"/>
       <c r="M5" s="23">
         <v>1.36</v>
       </c>
-      <c r="N5" s="44"/>
+      <c r="N5" s="53"/>
       <c r="O5" s="23">
         <v>1.32</v>
       </c>
-      <c r="P5" s="44"/>
+      <c r="P5" s="53"/>
       <c r="Q5" s="23">
         <v>1.26</v>
       </c>
@@ -40370,21 +40367,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="L2:L5"/>
+    <mergeCell ref="N2:N5"/>
+    <mergeCell ref="P2:P5"/>
     <mergeCell ref="H2:H5"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="J2:J5"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="M3:M4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="L2:L5"/>
-    <mergeCell ref="N2:N5"/>
-    <mergeCell ref="P2:P5"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B2:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -40411,65 +40408,65 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.4">
-      <c r="B3" s="43"/>
-      <c r="C3" s="48">
+      <c r="B3" s="52"/>
+      <c r="C3" s="59">
         <v>0</v>
       </c>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48">
+      <c r="D3" s="59"/>
+      <c r="E3" s="59">
         <v>5</v>
       </c>
-      <c r="F3" s="48"/>
-      <c r="G3" s="49">
+      <c r="F3" s="59"/>
+      <c r="G3" s="60">
         <v>10</v>
       </c>
-      <c r="H3" s="50"/>
-      <c r="I3" s="49">
+      <c r="H3" s="61"/>
+      <c r="I3" s="60">
         <v>15</v>
       </c>
-      <c r="J3" s="50"/>
-      <c r="K3" s="49">
+      <c r="J3" s="61"/>
+      <c r="K3" s="60">
         <v>20</v>
       </c>
-      <c r="L3" s="50"/>
-      <c r="M3" s="49">
+      <c r="L3" s="61"/>
+      <c r="M3" s="60">
         <v>25</v>
       </c>
-      <c r="N3" s="50"/>
-      <c r="O3" s="49">
+      <c r="N3" s="61"/>
+      <c r="O3" s="60">
         <v>30</v>
       </c>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="49">
+      <c r="P3" s="61"/>
+      <c r="Q3" s="60">
         <v>35</v>
       </c>
-      <c r="R3" s="50"/>
+      <c r="R3" s="61"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.4">
-      <c r="B4" s="44"/>
+      <c r="B4" s="53"/>
       <c r="C4" s="29" t="s">
         <v>13</v>
       </c>
@@ -41961,126 +41958,126 @@
   <cols>
     <col min="1" max="1" width="2.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.88671875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" style="62" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" style="41" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" style="12" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" style="62" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" style="41" customWidth="1"/>
     <col min="6" max="6" width="13.88671875" style="12" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" style="60" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" style="39" customWidth="1"/>
     <col min="8" max="8" width="13.88671875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" style="60" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" style="39" customWidth="1"/>
     <col min="10" max="10" width="13.88671875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.88671875" style="60" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" style="39" customWidth="1"/>
     <col min="12" max="12" width="13.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.88671875" style="60" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" style="39" customWidth="1"/>
     <col min="14" max="14" width="13.88671875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="13.88671875" style="60" customWidth="1"/>
+    <col min="15" max="15" width="13.88671875" style="39" customWidth="1"/>
     <col min="16" max="16" width="13.88671875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="13.88671875" style="60" customWidth="1"/>
+    <col min="17" max="17" width="13.88671875" style="39" customWidth="1"/>
     <col min="18" max="18" width="2.6640625" style="1" customWidth="1"/>
     <col min="19" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
     </row>
     <row r="3" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B3" s="48">
+      <c r="B3" s="59">
         <v>0</v>
       </c>
-      <c r="C3" s="48"/>
-      <c r="D3" s="49">
+      <c r="C3" s="59"/>
+      <c r="D3" s="60">
         <v>5</v>
       </c>
-      <c r="E3" s="50"/>
-      <c r="F3" s="49">
+      <c r="E3" s="61"/>
+      <c r="F3" s="60">
         <v>10</v>
       </c>
-      <c r="G3" s="50"/>
-      <c r="H3" s="49">
+      <c r="G3" s="61"/>
+      <c r="H3" s="60">
         <v>15</v>
       </c>
-      <c r="I3" s="50"/>
-      <c r="J3" s="49">
+      <c r="I3" s="61"/>
+      <c r="J3" s="60">
         <v>20</v>
       </c>
-      <c r="K3" s="50"/>
-      <c r="L3" s="49">
+      <c r="K3" s="61"/>
+      <c r="L3" s="60">
         <v>25</v>
       </c>
-      <c r="M3" s="50"/>
-      <c r="N3" s="49">
+      <c r="M3" s="61"/>
+      <c r="N3" s="60">
         <v>30</v>
       </c>
-      <c r="O3" s="50"/>
-      <c r="P3" s="49">
+      <c r="O3" s="61"/>
+      <c r="P3" s="60">
         <v>35</v>
       </c>
-      <c r="Q3" s="50"/>
+      <c r="Q3" s="61"/>
     </row>
     <row r="4" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="58" t="s">
+      <c r="C4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="58" t="s">
+      <c r="E4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="58" t="s">
+      <c r="G4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="58" t="s">
+      <c r="I4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="58" t="s">
+      <c r="K4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="L4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="58" t="s">
+      <c r="M4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="58" t="s">
+      <c r="O4" s="37" t="s">
         <v>16</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="Q4" s="58" t="s">
+      <c r="Q4" s="37" t="s">
         <v>16</v>
       </c>
     </row>
@@ -42116,7 +42113,7 @@
         <v>1.2</v>
       </c>
       <c r="C6" s="5">
-        <f t="shared" ref="C6:E15" si="0">LOG10(((2*1.4*B6^2-1.4+1)/(1.4+1)))</f>
+        <f t="shared" ref="C6:C15" si="0">LOG10(((2*1.4*B6^2-1.4+1)/(1.4+1)))</f>
         <v>0.1799345981374415</v>
       </c>
       <c r="D6" s="9">
@@ -42303,7 +42300,7 @@
         <f t="shared" si="0"/>
         <v>0.73878055848436919</v>
       </c>
-      <c r="D11" s="54">
+      <c r="D11" s="34">
         <v>1.24</v>
       </c>
       <c r="E11" s="18">
@@ -42342,7 +42339,7 @@
         <f t="shared" si="0"/>
         <v>0.8164622587764544</v>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="32">
         <v>1.3</v>
       </c>
       <c r="E12" s="17">
@@ -42351,7 +42348,7 @@
       <c r="F12" s="9">
         <v>1.5</v>
       </c>
-      <c r="G12" s="57">
+      <c r="G12" s="5">
         <v>0.222</v>
       </c>
       <c r="H12" s="9">
@@ -42391,13 +42388,13 @@
       <c r="E13" s="5">
         <v>0.45024910831936116</v>
       </c>
-      <c r="F13" s="54">
+      <c r="F13" s="34">
         <v>1.423</v>
       </c>
       <c r="G13" s="18">
         <v>0.26500000000000001</v>
       </c>
-      <c r="H13" s="54">
+      <c r="H13" s="34">
         <v>1.6140000000000001</v>
       </c>
       <c r="I13" s="18">
@@ -42434,10 +42431,10 @@
       <c r="E14" s="5">
         <v>0.55790802748270563</v>
       </c>
-      <c r="F14" s="55">
+      <c r="F14" s="35">
         <v>1.6</v>
       </c>
-      <c r="G14" s="56">
+      <c r="G14" s="36">
         <v>0.434</v>
       </c>
       <c r="H14" s="9">
@@ -42446,7 +42443,7 @@
       <c r="I14" s="5">
         <v>0.47</v>
       </c>
-      <c r="J14" s="54">
+      <c r="J14" s="34">
         <v>1.837</v>
       </c>
       <c r="K14" s="18">
@@ -42481,7 +42478,7 @@
       <c r="E15" s="5">
         <v>0.65321251377534373</v>
       </c>
-      <c r="F15" s="52">
+      <c r="F15" s="32">
         <v>1.8</v>
       </c>
       <c r="G15" s="17">
@@ -42523,13 +42520,13 @@
       <c r="E16" s="5">
         <v>0.73878055848436919</v>
       </c>
-      <c r="F16" s="51">
+      <c r="F16" s="31">
         <v>2.0070000000000001</v>
       </c>
       <c r="G16" s="16">
         <v>0.65321251377534373</v>
       </c>
-      <c r="H16" s="51">
+      <c r="H16" s="31">
         <v>2</v>
       </c>
       <c r="I16" s="16">
@@ -42571,7 +42568,7 @@
       <c r="G17" s="5">
         <v>0.73878055848436919</v>
       </c>
-      <c r="H17" s="52">
+      <c r="H17" s="32">
         <v>2.2000000000000002</v>
       </c>
       <c r="I17" s="17">
@@ -42583,7 +42580,7 @@
       <c r="K17" s="5">
         <v>0.74</v>
       </c>
-      <c r="L17" s="54">
+      <c r="L17" s="34">
         <v>2.1219999999999999</v>
       </c>
       <c r="M17" s="18">
@@ -42617,13 +42614,13 @@
       <c r="G18" s="5">
         <v>0.8164622587764544</v>
       </c>
-      <c r="H18" s="51">
+      <c r="H18" s="31">
         <v>2.4159999999999999</v>
       </c>
       <c r="I18" s="16">
         <v>0.8164622587764544</v>
       </c>
-      <c r="J18" s="52">
+      <c r="J18" s="32">
         <v>2.4</v>
       </c>
       <c r="K18" s="17">
@@ -42635,7 +42632,7 @@
       <c r="M18" s="5">
         <v>0.68799999999999994</v>
       </c>
-      <c r="N18" s="54">
+      <c r="N18" s="34">
         <v>2.5179999999999998</v>
       </c>
       <c r="O18" s="18">
@@ -42649,7 +42646,7 @@
       </c>
     </row>
     <row r="19" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B19" s="53"/>
+      <c r="B19" s="33"/>
       <c r="C19" s="13"/>
       <c r="D19" s="9">
         <v>2.8039999999999998</v>
@@ -42669,7 +42666,7 @@
       <c r="I19" s="5">
         <v>0.88761730033573627</v>
       </c>
-      <c r="J19" s="51">
+      <c r="J19" s="31">
         <v>2.63</v>
       </c>
       <c r="K19" s="16">
@@ -42695,7 +42692,7 @@
       </c>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B20" s="53"/>
+      <c r="B20" s="33"/>
       <c r="C20" s="13"/>
       <c r="D20" s="9">
         <v>3.004</v>
@@ -42709,13 +42706,13 @@
       <c r="G20" s="5">
         <v>0.95327633666730427</v>
       </c>
-      <c r="H20" s="51">
+      <c r="H20" s="31">
         <v>2.8159999999999998</v>
       </c>
       <c r="I20" s="5">
         <v>0.95327633666730427</v>
       </c>
-      <c r="J20" s="51">
+      <c r="J20" s="31">
         <v>2.83</v>
       </c>
       <c r="K20" s="5">
@@ -42733,7 +42730,7 @@
       <c r="O20" s="5">
         <v>0.89800000000000002</v>
       </c>
-      <c r="P20" s="54">
+      <c r="P20" s="34">
         <v>3.14</v>
       </c>
       <c r="Q20" s="18">
@@ -42741,7 +42738,7 @@
       </c>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B21" s="53"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="13"/>
       <c r="D21" s="9"/>
       <c r="E21" s="5"/>
@@ -42784,665 +42781,665 @@
     </row>
     <row r="22" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B22"/>
-      <c r="C22" s="59"/>
+      <c r="C22" s="38"/>
       <c r="D22"/>
-      <c r="E22" s="59"/>
+      <c r="E22" s="38"/>
       <c r="F22"/>
-      <c r="G22" s="59"/>
+      <c r="G22" s="38"/>
       <c r="H22"/>
-      <c r="I22" s="59"/>
+      <c r="I22" s="38"/>
       <c r="J22"/>
-      <c r="K22" s="59"/>
+      <c r="K22" s="38"/>
       <c r="L22"/>
-      <c r="M22" s="59"/>
+      <c r="M22" s="38"/>
       <c r="N22"/>
-      <c r="O22" s="59"/>
+      <c r="O22" s="38"/>
       <c r="P22"/>
-      <c r="Q22" s="59"/>
+      <c r="Q22" s="38"/>
     </row>
     <row r="23" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B23"/>
-      <c r="C23" s="59"/>
+      <c r="C23" s="38"/>
       <c r="D23"/>
-      <c r="E23" s="59"/>
+      <c r="E23" s="38"/>
       <c r="F23"/>
-      <c r="G23" s="59"/>
+      <c r="G23" s="38"/>
       <c r="H23"/>
-      <c r="I23" s="59"/>
+      <c r="I23" s="38"/>
       <c r="J23"/>
-      <c r="K23" s="59"/>
+      <c r="K23" s="38"/>
       <c r="L23"/>
-      <c r="M23" s="59"/>
+      <c r="M23" s="38"/>
       <c r="N23"/>
-      <c r="O23" s="59"/>
+      <c r="O23" s="38"/>
       <c r="P23"/>
-      <c r="Q23" s="59"/>
+      <c r="Q23" s="38"/>
     </row>
     <row r="24" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B24"/>
-      <c r="C24" s="59"/>
+      <c r="C24" s="38"/>
       <c r="D24"/>
-      <c r="E24" s="59"/>
+      <c r="E24" s="38"/>
       <c r="F24"/>
-      <c r="G24" s="59"/>
+      <c r="G24" s="38"/>
       <c r="H24"/>
-      <c r="I24" s="59"/>
+      <c r="I24" s="38"/>
       <c r="J24"/>
-      <c r="K24" s="59"/>
+      <c r="K24" s="38"/>
       <c r="L24"/>
-      <c r="M24" s="59"/>
+      <c r="M24" s="38"/>
       <c r="N24"/>
-      <c r="O24" s="59"/>
+      <c r="O24" s="38"/>
       <c r="P24"/>
-      <c r="Q24" s="59"/>
+      <c r="Q24" s="38"/>
     </row>
     <row r="25" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B25"/>
-      <c r="C25" s="59"/>
+      <c r="C25" s="38"/>
       <c r="D25"/>
-      <c r="E25" s="59"/>
+      <c r="E25" s="38"/>
       <c r="F25"/>
-      <c r="G25" s="59"/>
+      <c r="G25" s="38"/>
       <c r="H25"/>
-      <c r="I25" s="59"/>
+      <c r="I25" s="38"/>
       <c r="J25"/>
-      <c r="K25" s="59"/>
+      <c r="K25" s="38"/>
       <c r="L25"/>
-      <c r="M25" s="59"/>
+      <c r="M25" s="38"/>
       <c r="N25"/>
-      <c r="O25" s="59"/>
+      <c r="O25" s="38"/>
       <c r="P25"/>
-      <c r="Q25" s="59"/>
+      <c r="Q25" s="38"/>
     </row>
     <row r="26" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B26"/>
-      <c r="C26" s="59"/>
+      <c r="C26" s="38"/>
       <c r="D26"/>
-      <c r="E26" s="59"/>
+      <c r="E26" s="38"/>
       <c r="F26"/>
-      <c r="G26" s="59"/>
+      <c r="G26" s="38"/>
       <c r="H26"/>
-      <c r="I26" s="59"/>
+      <c r="I26" s="38"/>
       <c r="J26"/>
-      <c r="K26" s="59"/>
+      <c r="K26" s="38"/>
       <c r="L26"/>
-      <c r="M26" s="59"/>
+      <c r="M26" s="38"/>
       <c r="N26"/>
-      <c r="O26" s="59"/>
+      <c r="O26" s="38"/>
       <c r="P26"/>
-      <c r="Q26" s="59"/>
+      <c r="Q26" s="38"/>
     </row>
     <row r="27" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B27"/>
-      <c r="C27" s="59"/>
+      <c r="C27" s="38"/>
       <c r="D27"/>
-      <c r="E27" s="59"/>
+      <c r="E27" s="38"/>
       <c r="F27"/>
-      <c r="G27" s="59"/>
+      <c r="G27" s="38"/>
       <c r="H27"/>
-      <c r="I27" s="59"/>
+      <c r="I27" s="38"/>
       <c r="J27"/>
-      <c r="K27" s="59"/>
+      <c r="K27" s="38"/>
       <c r="L27"/>
-      <c r="M27" s="59"/>
+      <c r="M27" s="38"/>
       <c r="N27"/>
-      <c r="O27" s="59"/>
+      <c r="O27" s="38"/>
       <c r="P27"/>
-      <c r="Q27" s="59"/>
+      <c r="Q27" s="38"/>
     </row>
     <row r="28" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B28"/>
-      <c r="C28" s="59"/>
+      <c r="C28" s="38"/>
       <c r="D28"/>
-      <c r="E28" s="59"/>
+      <c r="E28" s="38"/>
       <c r="F28"/>
-      <c r="G28" s="59"/>
+      <c r="G28" s="38"/>
       <c r="H28"/>
-      <c r="I28" s="59"/>
+      <c r="I28" s="38"/>
       <c r="J28"/>
-      <c r="K28" s="59"/>
+      <c r="K28" s="38"/>
       <c r="L28"/>
-      <c r="M28" s="59"/>
+      <c r="M28" s="38"/>
       <c r="N28"/>
-      <c r="O28" s="59"/>
+      <c r="O28" s="38"/>
       <c r="P28"/>
-      <c r="Q28" s="59"/>
+      <c r="Q28" s="38"/>
     </row>
     <row r="29" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B29"/>
-      <c r="C29" s="59"/>
+      <c r="C29" s="38"/>
       <c r="D29"/>
-      <c r="E29" s="59"/>
+      <c r="E29" s="38"/>
       <c r="F29"/>
-      <c r="G29" s="59"/>
+      <c r="G29" s="38"/>
       <c r="H29"/>
-      <c r="I29" s="59"/>
+      <c r="I29" s="38"/>
       <c r="J29"/>
-      <c r="K29" s="59"/>
+      <c r="K29" s="38"/>
       <c r="L29"/>
-      <c r="M29" s="59"/>
+      <c r="M29" s="38"/>
       <c r="N29"/>
-      <c r="O29" s="59"/>
+      <c r="O29" s="38"/>
       <c r="P29"/>
-      <c r="Q29" s="59"/>
+      <c r="Q29" s="38"/>
       <c r="AB29"/>
     </row>
     <row r="30" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B30"/>
-      <c r="C30" s="59"/>
+      <c r="C30" s="38"/>
       <c r="D30"/>
-      <c r="E30" s="59"/>
+      <c r="E30" s="38"/>
       <c r="F30"/>
-      <c r="G30" s="59"/>
+      <c r="G30" s="38"/>
       <c r="H30"/>
-      <c r="I30" s="59"/>
+      <c r="I30" s="38"/>
       <c r="J30"/>
-      <c r="K30" s="59"/>
+      <c r="K30" s="38"/>
       <c r="L30"/>
-      <c r="M30" s="59"/>
+      <c r="M30" s="38"/>
       <c r="N30"/>
-      <c r="O30" s="59"/>
+      <c r="O30" s="38"/>
       <c r="P30"/>
-      <c r="Q30" s="59"/>
+      <c r="Q30" s="38"/>
     </row>
     <row r="31" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B31"/>
-      <c r="C31" s="59"/>
+      <c r="C31" s="38"/>
       <c r="D31"/>
-      <c r="E31" s="59"/>
+      <c r="E31" s="38"/>
       <c r="F31"/>
-      <c r="G31" s="59"/>
+      <c r="G31" s="38"/>
       <c r="H31"/>
-      <c r="I31" s="59"/>
+      <c r="I31" s="38"/>
       <c r="J31"/>
-      <c r="K31" s="59"/>
+      <c r="K31" s="38"/>
       <c r="L31"/>
-      <c r="M31" s="59"/>
+      <c r="M31" s="38"/>
       <c r="N31"/>
-      <c r="O31" s="59"/>
+      <c r="O31" s="38"/>
       <c r="P31"/>
-      <c r="Q31" s="59"/>
+      <c r="Q31" s="38"/>
     </row>
     <row r="32" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B32"/>
-      <c r="C32" s="59"/>
+      <c r="C32" s="38"/>
       <c r="D32"/>
-      <c r="E32" s="59"/>
+      <c r="E32" s="38"/>
       <c r="F32"/>
-      <c r="G32" s="59"/>
+      <c r="G32" s="38"/>
       <c r="H32"/>
-      <c r="I32" s="59"/>
+      <c r="I32" s="38"/>
       <c r="J32"/>
-      <c r="K32" s="59"/>
+      <c r="K32" s="38"/>
       <c r="L32"/>
-      <c r="M32" s="59"/>
+      <c r="M32" s="38"/>
       <c r="N32"/>
-      <c r="O32" s="59"/>
+      <c r="O32" s="38"/>
       <c r="P32"/>
-      <c r="Q32" s="59"/>
+      <c r="Q32" s="38"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B33"/>
-      <c r="C33" s="59"/>
+      <c r="C33" s="38"/>
       <c r="D33"/>
-      <c r="E33" s="59"/>
+      <c r="E33" s="38"/>
       <c r="F33"/>
-      <c r="G33" s="59"/>
+      <c r="G33" s="38"/>
       <c r="H33"/>
-      <c r="I33" s="59"/>
+      <c r="I33" s="38"/>
       <c r="J33"/>
-      <c r="K33" s="59"/>
+      <c r="K33" s="38"/>
       <c r="L33"/>
-      <c r="M33" s="59"/>
+      <c r="M33" s="38"/>
       <c r="N33"/>
-      <c r="O33" s="59"/>
+      <c r="O33" s="38"/>
       <c r="P33"/>
-      <c r="Q33" s="59"/>
+      <c r="Q33" s="38"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B34"/>
-      <c r="C34" s="59"/>
+      <c r="C34" s="38"/>
       <c r="D34"/>
-      <c r="E34" s="59"/>
+      <c r="E34" s="38"/>
       <c r="F34"/>
-      <c r="G34" s="59"/>
+      <c r="G34" s="38"/>
       <c r="H34"/>
-      <c r="I34" s="59"/>
+      <c r="I34" s="38"/>
       <c r="J34"/>
-      <c r="K34" s="59"/>
+      <c r="K34" s="38"/>
       <c r="L34"/>
-      <c r="M34" s="59"/>
+      <c r="M34" s="38"/>
       <c r="N34"/>
-      <c r="O34" s="59"/>
+      <c r="O34" s="38"/>
       <c r="P34"/>
-      <c r="Q34" s="59"/>
+      <c r="Q34" s="38"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B35"/>
-      <c r="C35" s="59"/>
+      <c r="C35" s="38"/>
       <c r="D35"/>
-      <c r="E35" s="59"/>
+      <c r="E35" s="38"/>
       <c r="F35"/>
-      <c r="G35" s="59"/>
+      <c r="G35" s="38"/>
       <c r="H35"/>
-      <c r="I35" s="59"/>
+      <c r="I35" s="38"/>
       <c r="J35"/>
-      <c r="K35" s="59"/>
+      <c r="K35" s="38"/>
       <c r="L35"/>
-      <c r="M35" s="59"/>
+      <c r="M35" s="38"/>
       <c r="N35"/>
-      <c r="O35" s="59"/>
+      <c r="O35" s="38"/>
       <c r="P35"/>
-      <c r="Q35" s="59"/>
+      <c r="Q35" s="38"/>
     </row>
     <row r="36" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B36"/>
-      <c r="C36" s="59"/>
+      <c r="C36" s="38"/>
       <c r="D36"/>
-      <c r="E36" s="59"/>
+      <c r="E36" s="38"/>
       <c r="F36"/>
-      <c r="G36" s="59"/>
+      <c r="G36" s="38"/>
       <c r="H36"/>
-      <c r="I36" s="59"/>
+      <c r="I36" s="38"/>
       <c r="J36"/>
-      <c r="K36" s="59"/>
+      <c r="K36" s="38"/>
       <c r="L36"/>
-      <c r="M36" s="59"/>
+      <c r="M36" s="38"/>
       <c r="N36"/>
-      <c r="O36" s="59"/>
+      <c r="O36" s="38"/>
       <c r="P36"/>
-      <c r="Q36" s="59"/>
+      <c r="Q36" s="38"/>
     </row>
     <row r="37" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B37"/>
-      <c r="C37" s="59"/>
+      <c r="C37" s="38"/>
       <c r="D37"/>
-      <c r="E37" s="59"/>
+      <c r="E37" s="38"/>
       <c r="F37"/>
-      <c r="G37" s="59"/>
+      <c r="G37" s="38"/>
       <c r="H37"/>
-      <c r="I37" s="59"/>
+      <c r="I37" s="38"/>
       <c r="J37"/>
-      <c r="K37" s="59"/>
+      <c r="K37" s="38"/>
       <c r="L37"/>
-      <c r="M37" s="59"/>
+      <c r="M37" s="38"/>
       <c r="N37"/>
-      <c r="O37" s="59"/>
+      <c r="O37" s="38"/>
       <c r="P37"/>
-      <c r="Q37" s="59"/>
+      <c r="Q37" s="38"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B38"/>
-      <c r="C38" s="59"/>
+      <c r="C38" s="38"/>
       <c r="D38"/>
-      <c r="E38" s="59"/>
+      <c r="E38" s="38"/>
       <c r="F38"/>
-      <c r="G38" s="59"/>
+      <c r="G38" s="38"/>
       <c r="H38"/>
-      <c r="I38" s="59"/>
+      <c r="I38" s="38"/>
       <c r="J38"/>
-      <c r="K38" s="59"/>
+      <c r="K38" s="38"/>
       <c r="L38"/>
-      <c r="M38" s="59"/>
+      <c r="M38" s="38"/>
       <c r="N38"/>
-      <c r="O38" s="59"/>
+      <c r="O38" s="38"/>
       <c r="P38"/>
-      <c r="Q38" s="59"/>
+      <c r="Q38" s="38"/>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B39"/>
-      <c r="C39" s="59"/>
+      <c r="C39" s="38"/>
       <c r="D39"/>
-      <c r="E39" s="59"/>
+      <c r="E39" s="38"/>
       <c r="F39"/>
-      <c r="G39" s="59"/>
+      <c r="G39" s="38"/>
       <c r="H39"/>
-      <c r="I39" s="59"/>
+      <c r="I39" s="38"/>
       <c r="J39"/>
-      <c r="K39" s="59"/>
+      <c r="K39" s="38"/>
       <c r="L39"/>
-      <c r="M39" s="59"/>
+      <c r="M39" s="38"/>
       <c r="N39"/>
-      <c r="O39" s="59"/>
+      <c r="O39" s="38"/>
       <c r="P39"/>
-      <c r="Q39" s="59"/>
+      <c r="Q39" s="38"/>
     </row>
     <row r="40" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B40"/>
-      <c r="C40" s="59"/>
+      <c r="C40" s="38"/>
       <c r="D40"/>
-      <c r="E40" s="59"/>
+      <c r="E40" s="38"/>
       <c r="F40"/>
-      <c r="G40" s="59"/>
+      <c r="G40" s="38"/>
       <c r="H40"/>
-      <c r="I40" s="59"/>
+      <c r="I40" s="38"/>
       <c r="J40"/>
-      <c r="K40" s="59"/>
+      <c r="K40" s="38"/>
       <c r="L40"/>
-      <c r="M40" s="59"/>
+      <c r="M40" s="38"/>
       <c r="N40"/>
-      <c r="O40" s="59"/>
+      <c r="O40" s="38"/>
       <c r="P40"/>
-      <c r="Q40" s="59"/>
+      <c r="Q40" s="38"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B41"/>
-      <c r="C41" s="59"/>
+      <c r="C41" s="38"/>
       <c r="D41"/>
-      <c r="E41" s="59"/>
+      <c r="E41" s="38"/>
       <c r="F41"/>
-      <c r="G41" s="59"/>
+      <c r="G41" s="38"/>
       <c r="H41"/>
-      <c r="I41" s="59"/>
+      <c r="I41" s="38"/>
       <c r="J41"/>
-      <c r="K41" s="59"/>
+      <c r="K41" s="38"/>
       <c r="L41"/>
-      <c r="M41" s="59"/>
+      <c r="M41" s="38"/>
       <c r="N41"/>
-      <c r="O41" s="59"/>
+      <c r="O41" s="38"/>
       <c r="P41"/>
-      <c r="Q41" s="59"/>
+      <c r="Q41" s="38"/>
     </row>
     <row r="42" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B42"/>
-      <c r="C42" s="59"/>
+      <c r="C42" s="38"/>
       <c r="D42"/>
-      <c r="E42" s="59"/>
+      <c r="E42" s="38"/>
       <c r="F42"/>
-      <c r="G42" s="59"/>
+      <c r="G42" s="38"/>
       <c r="H42"/>
-      <c r="I42" s="59"/>
+      <c r="I42" s="38"/>
       <c r="J42"/>
-      <c r="K42" s="59"/>
+      <c r="K42" s="38"/>
       <c r="L42"/>
-      <c r="M42" s="59"/>
+      <c r="M42" s="38"/>
       <c r="N42"/>
-      <c r="O42" s="59"/>
+      <c r="O42" s="38"/>
       <c r="P42"/>
-      <c r="Q42" s="59"/>
+      <c r="Q42" s="38"/>
     </row>
     <row r="43" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B43"/>
-      <c r="C43" s="59"/>
+      <c r="C43" s="38"/>
       <c r="D43"/>
-      <c r="E43" s="59"/>
+      <c r="E43" s="38"/>
       <c r="F43"/>
-      <c r="G43" s="59"/>
+      <c r="G43" s="38"/>
       <c r="H43"/>
-      <c r="I43" s="59"/>
+      <c r="I43" s="38"/>
       <c r="J43"/>
-      <c r="K43" s="59"/>
+      <c r="K43" s="38"/>
       <c r="L43"/>
-      <c r="M43" s="59"/>
+      <c r="M43" s="38"/>
       <c r="N43"/>
-      <c r="O43" s="59"/>
+      <c r="O43" s="38"/>
       <c r="P43"/>
-      <c r="Q43" s="59"/>
+      <c r="Q43" s="38"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B44"/>
-      <c r="C44" s="59"/>
+      <c r="C44" s="38"/>
       <c r="D44"/>
-      <c r="E44" s="59"/>
+      <c r="E44" s="38"/>
       <c r="F44"/>
-      <c r="G44" s="59"/>
+      <c r="G44" s="38"/>
       <c r="H44"/>
-      <c r="I44" s="59"/>
+      <c r="I44" s="38"/>
       <c r="J44"/>
-      <c r="K44" s="59"/>
+      <c r="K44" s="38"/>
       <c r="L44"/>
-      <c r="M44" s="59"/>
+      <c r="M44" s="38"/>
       <c r="N44"/>
-      <c r="O44" s="59"/>
+      <c r="O44" s="38"/>
       <c r="P44"/>
-      <c r="Q44" s="59"/>
+      <c r="Q44" s="38"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B45"/>
-      <c r="C45" s="59"/>
+      <c r="C45" s="38"/>
       <c r="D45"/>
-      <c r="E45" s="59"/>
+      <c r="E45" s="38"/>
       <c r="F45"/>
-      <c r="G45" s="59"/>
+      <c r="G45" s="38"/>
       <c r="H45"/>
-      <c r="I45" s="59"/>
+      <c r="I45" s="38"/>
       <c r="J45"/>
-      <c r="K45" s="59"/>
+      <c r="K45" s="38"/>
       <c r="L45"/>
-      <c r="M45" s="59"/>
+      <c r="M45" s="38"/>
       <c r="N45"/>
-      <c r="O45" s="59"/>
+      <c r="O45" s="38"/>
       <c r="P45"/>
-      <c r="Q45" s="59"/>
+      <c r="Q45" s="38"/>
     </row>
     <row r="46" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B46"/>
-      <c r="C46" s="59"/>
+      <c r="C46" s="38"/>
       <c r="D46"/>
-      <c r="E46" s="59"/>
+      <c r="E46" s="38"/>
       <c r="F46"/>
-      <c r="G46" s="59"/>
+      <c r="G46" s="38"/>
       <c r="H46"/>
-      <c r="I46" s="59"/>
+      <c r="I46" s="38"/>
       <c r="J46"/>
-      <c r="K46" s="59"/>
+      <c r="K46" s="38"/>
       <c r="L46"/>
-      <c r="M46" s="59"/>
+      <c r="M46" s="38"/>
       <c r="N46"/>
-      <c r="O46" s="59"/>
+      <c r="O46" s="38"/>
       <c r="P46"/>
-      <c r="Q46" s="59"/>
+      <c r="Q46" s="38"/>
     </row>
     <row r="47" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B47"/>
-      <c r="C47" s="59"/>
+      <c r="C47" s="38"/>
       <c r="D47"/>
-      <c r="E47" s="59"/>
+      <c r="E47" s="38"/>
       <c r="F47"/>
-      <c r="G47" s="59"/>
+      <c r="G47" s="38"/>
       <c r="H47"/>
-      <c r="I47" s="59"/>
+      <c r="I47" s="38"/>
       <c r="J47"/>
-      <c r="K47" s="59"/>
+      <c r="K47" s="38"/>
       <c r="L47"/>
-      <c r="M47" s="59"/>
+      <c r="M47" s="38"/>
       <c r="N47"/>
-      <c r="O47" s="59"/>
+      <c r="O47" s="38"/>
       <c r="P47"/>
-      <c r="Q47" s="59"/>
+      <c r="Q47" s="38"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B48"/>
-      <c r="C48" s="59"/>
+      <c r="C48" s="38"/>
       <c r="D48"/>
-      <c r="E48" s="59"/>
+      <c r="E48" s="38"/>
       <c r="F48"/>
-      <c r="G48" s="59"/>
+      <c r="G48" s="38"/>
       <c r="H48"/>
-      <c r="I48" s="59"/>
+      <c r="I48" s="38"/>
       <c r="J48"/>
-      <c r="K48" s="59"/>
+      <c r="K48" s="38"/>
       <c r="L48"/>
-      <c r="M48" s="59"/>
+      <c r="M48" s="38"/>
       <c r="N48"/>
-      <c r="O48" s="59"/>
+      <c r="O48" s="38"/>
       <c r="P48"/>
-      <c r="Q48" s="59"/>
+      <c r="Q48" s="38"/>
     </row>
     <row r="49" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B49"/>
-      <c r="C49" s="59"/>
+      <c r="C49" s="38"/>
       <c r="D49"/>
-      <c r="E49" s="59"/>
+      <c r="E49" s="38"/>
       <c r="F49"/>
-      <c r="G49" s="59"/>
+      <c r="G49" s="38"/>
       <c r="H49"/>
-      <c r="I49" s="59"/>
+      <c r="I49" s="38"/>
       <c r="J49"/>
-      <c r="K49" s="59"/>
+      <c r="K49" s="38"/>
       <c r="L49"/>
-      <c r="M49" s="59"/>
+      <c r="M49" s="38"/>
       <c r="N49"/>
-      <c r="O49" s="59"/>
+      <c r="O49" s="38"/>
       <c r="P49"/>
-      <c r="Q49" s="59"/>
+      <c r="Q49" s="38"/>
     </row>
     <row r="50" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B50"/>
-      <c r="C50" s="59"/>
+      <c r="C50" s="38"/>
       <c r="D50"/>
-      <c r="E50" s="59"/>
+      <c r="E50" s="38"/>
       <c r="F50"/>
-      <c r="G50" s="59"/>
+      <c r="G50" s="38"/>
       <c r="H50"/>
-      <c r="I50" s="59"/>
+      <c r="I50" s="38"/>
       <c r="J50"/>
-      <c r="K50" s="59"/>
+      <c r="K50" s="38"/>
       <c r="L50"/>
-      <c r="M50" s="59"/>
+      <c r="M50" s="38"/>
       <c r="N50"/>
-      <c r="O50" s="59"/>
+      <c r="O50" s="38"/>
       <c r="P50"/>
-      <c r="Q50" s="59"/>
+      <c r="Q50" s="38"/>
     </row>
     <row r="51" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B51"/>
-      <c r="C51" s="59"/>
+      <c r="C51" s="38"/>
       <c r="D51"/>
-      <c r="E51" s="59"/>
+      <c r="E51" s="38"/>
       <c r="F51"/>
-      <c r="G51" s="59"/>
+      <c r="G51" s="38"/>
       <c r="H51"/>
-      <c r="I51" s="59"/>
+      <c r="I51" s="38"/>
       <c r="J51"/>
-      <c r="K51" s="59"/>
+      <c r="K51" s="38"/>
       <c r="L51"/>
-      <c r="M51" s="59"/>
+      <c r="M51" s="38"/>
       <c r="N51"/>
-      <c r="O51" s="59"/>
+      <c r="O51" s="38"/>
       <c r="P51"/>
-      <c r="Q51" s="59"/>
+      <c r="Q51" s="38"/>
     </row>
     <row r="52" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B52"/>
-      <c r="C52" s="59"/>
+      <c r="C52" s="38"/>
       <c r="D52"/>
-      <c r="E52" s="59"/>
+      <c r="E52" s="38"/>
       <c r="F52"/>
-      <c r="G52" s="59"/>
+      <c r="G52" s="38"/>
       <c r="H52"/>
-      <c r="I52" s="59"/>
+      <c r="I52" s="38"/>
       <c r="J52"/>
-      <c r="K52" s="59"/>
+      <c r="K52" s="38"/>
       <c r="L52"/>
-      <c r="M52" s="59"/>
+      <c r="M52" s="38"/>
       <c r="N52"/>
-      <c r="O52" s="59"/>
+      <c r="O52" s="38"/>
       <c r="P52"/>
-      <c r="Q52" s="59"/>
+      <c r="Q52" s="38"/>
     </row>
     <row r="53" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C53" s="59"/>
-      <c r="E53" s="59"/>
-      <c r="G53" s="59"/>
-      <c r="I53" s="59"/>
-      <c r="K53" s="59"/>
-      <c r="M53" s="59"/>
-      <c r="O53" s="59"/>
-      <c r="Q53" s="59"/>
+      <c r="C53" s="38"/>
+      <c r="E53" s="38"/>
+      <c r="G53" s="38"/>
+      <c r="I53" s="38"/>
+      <c r="K53" s="38"/>
+      <c r="M53" s="38"/>
+      <c r="O53" s="38"/>
+      <c r="Q53" s="38"/>
     </row>
     <row r="54" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C54" s="59"/>
-      <c r="E54" s="59"/>
-      <c r="G54" s="59"/>
-      <c r="I54" s="59"/>
-      <c r="K54" s="59"/>
-      <c r="M54" s="59"/>
-      <c r="O54" s="59"/>
-      <c r="Q54" s="59"/>
+      <c r="C54" s="38"/>
+      <c r="E54" s="38"/>
+      <c r="G54" s="38"/>
+      <c r="I54" s="38"/>
+      <c r="K54" s="38"/>
+      <c r="M54" s="38"/>
+      <c r="O54" s="38"/>
+      <c r="Q54" s="38"/>
     </row>
     <row r="55" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C55" s="59"/>
-      <c r="E55" s="59"/>
-      <c r="G55" s="59"/>
-      <c r="I55" s="59"/>
-      <c r="K55" s="59"/>
-      <c r="M55" s="59"/>
-      <c r="O55" s="59"/>
-      <c r="Q55" s="59"/>
+      <c r="C55" s="38"/>
+      <c r="E55" s="38"/>
+      <c r="G55" s="38"/>
+      <c r="I55" s="38"/>
+      <c r="K55" s="38"/>
+      <c r="M55" s="38"/>
+      <c r="O55" s="38"/>
+      <c r="Q55" s="38"/>
     </row>
     <row r="56" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C56" s="59"/>
-      <c r="E56" s="59"/>
-      <c r="G56" s="59"/>
-      <c r="I56" s="59"/>
-      <c r="K56" s="59"/>
-      <c r="M56" s="59"/>
-      <c r="O56" s="59"/>
-      <c r="Q56" s="59"/>
+      <c r="C56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="G56" s="38"/>
+      <c r="I56" s="38"/>
+      <c r="K56" s="38"/>
+      <c r="M56" s="38"/>
+      <c r="O56" s="38"/>
+      <c r="Q56" s="38"/>
     </row>
     <row r="57" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C57" s="59"/>
-      <c r="E57" s="59"/>
-      <c r="G57" s="59"/>
-      <c r="I57" s="59"/>
-      <c r="K57" s="59"/>
-      <c r="M57" s="59"/>
-      <c r="O57" s="59"/>
-      <c r="Q57" s="59"/>
+      <c r="C57" s="38"/>
+      <c r="E57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="I57" s="38"/>
+      <c r="K57" s="38"/>
+      <c r="M57" s="38"/>
+      <c r="O57" s="38"/>
+      <c r="Q57" s="38"/>
     </row>
     <row r="58" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C58" s="59"/>
-      <c r="E58" s="59"/>
-      <c r="G58" s="59"/>
-      <c r="I58" s="59"/>
-      <c r="K58" s="59"/>
-      <c r="M58" s="59"/>
-      <c r="O58" s="59"/>
-      <c r="Q58" s="59"/>
+      <c r="C58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="G58" s="38"/>
+      <c r="I58" s="38"/>
+      <c r="K58" s="38"/>
+      <c r="M58" s="38"/>
+      <c r="O58" s="38"/>
+      <c r="Q58" s="38"/>
     </row>
     <row r="59" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C59" s="59"/>
-      <c r="E59" s="59"/>
-      <c r="G59" s="59"/>
-      <c r="I59" s="59"/>
-      <c r="K59" s="59"/>
-      <c r="M59" s="59"/>
-      <c r="O59" s="59"/>
-      <c r="Q59" s="59"/>
+      <c r="C59" s="38"/>
+      <c r="E59" s="38"/>
+      <c r="G59" s="38"/>
+      <c r="I59" s="38"/>
+      <c r="K59" s="38"/>
+      <c r="M59" s="38"/>
+      <c r="O59" s="38"/>
+      <c r="Q59" s="38"/>
     </row>
     <row r="60" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C60" s="59"/>
-      <c r="E60" s="59"/>
-      <c r="G60" s="59"/>
-      <c r="I60" s="59"/>
-      <c r="K60" s="59"/>
-      <c r="M60" s="59"/>
-      <c r="O60" s="59"/>
-      <c r="Q60" s="59"/>
+      <c r="C60" s="38"/>
+      <c r="E60" s="38"/>
+      <c r="G60" s="38"/>
+      <c r="I60" s="38"/>
+      <c r="K60" s="38"/>
+      <c r="M60" s="38"/>
+      <c r="O60" s="38"/>
+      <c r="Q60" s="38"/>
     </row>
     <row r="61" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C61" s="59"/>
-      <c r="E61" s="59"/>
-      <c r="G61" s="59"/>
-      <c r="I61" s="59"/>
-      <c r="K61" s="59"/>
-      <c r="M61" s="59"/>
-      <c r="O61" s="59"/>
-      <c r="Q61" s="59"/>
+      <c r="C61" s="38"/>
+      <c r="E61" s="38"/>
+      <c r="G61" s="38"/>
+      <c r="I61" s="38"/>
+      <c r="K61" s="38"/>
+      <c r="M61" s="38"/>
+      <c r="O61" s="38"/>
+      <c r="Q61" s="38"/>
     </row>
     <row r="62" spans="2:17" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B62" s="30"/>
-      <c r="C62" s="61"/>
+      <c r="C62" s="40"/>
       <c r="D62" s="30"/>
-      <c r="E62" s="61"/>
+      <c r="E62" s="40"/>
       <c r="F62" s="30"/>
-      <c r="G62" s="59"/>
-      <c r="I62" s="59"/>
-      <c r="K62" s="59"/>
-      <c r="M62" s="59"/>
-      <c r="O62" s="59"/>
-      <c r="Q62" s="59"/>
+      <c r="G62" s="38"/>
+      <c r="I62" s="38"/>
+      <c r="K62" s="38"/>
+      <c r="M62" s="38"/>
+      <c r="O62" s="38"/>
+      <c r="Q62" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>